<commit_message>
v0.2.3 - gantt updated
</commit_message>
<xml_diff>
--- a/docs/fattibilita/template_gantt.xlsx
+++ b/docs/fattibilita/template_gantt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9125bfcb271df092/Documenti/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="438" documentId="13_ncr:1_{E57995CB-B28B-4041-9AE6-B60AE61FECF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A566A0EC-CC84-4800-A6EF-4B6E2AE666E8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F394920-092C-4BAA-9FF9-1472E0680BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9327F8D6-4F37-4E25-8083-20A17765DC2F}"/>
   </bookViews>
@@ -638,6 +638,18 @@
     <xf numFmtId="166" fontId="0" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -646,18 +658,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -719,10 +719,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1058,78 +1054,78 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:47" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="58"/>
+      <c r="D2" s="62"/>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="3:47" x14ac:dyDescent="0.3">
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="64"/>
+      <c r="D3" s="61"/>
       <c r="H3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="61" t="str">
+      <c r="I3" s="58" t="str">
         <f>TEXT(I5,"MMM")</f>
         <v>Oct</v>
       </c>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
-      <c r="M3" s="61" t="str">
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="58" t="str">
         <f>TEXT(M5,"MMM")</f>
         <v>Nov</v>
       </c>
-      <c r="N3" s="62"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="63"/>
-      <c r="Q3" s="61" t="str">
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="58" t="str">
         <f>TEXT(Q5,"MMM")</f>
         <v>Dec</v>
       </c>
-      <c r="R3" s="62"/>
-      <c r="S3" s="62"/>
-      <c r="T3" s="62"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
       <c r="U3" s="7"/>
-      <c r="V3" s="61" t="str">
+      <c r="V3" s="58" t="str">
         <f>TEXT(V5,"MMM")</f>
         <v>Jan</v>
       </c>
-      <c r="W3" s="62"/>
-      <c r="X3" s="62"/>
-      <c r="Y3" s="63"/>
-      <c r="Z3" s="61" t="str">
+      <c r="W3" s="59"/>
+      <c r="X3" s="59"/>
+      <c r="Y3" s="60"/>
+      <c r="Z3" s="58" t="str">
         <f>TEXT(Z5,"MMM")</f>
         <v>Feb</v>
       </c>
-      <c r="AA3" s="62"/>
-      <c r="AB3" s="62"/>
-      <c r="AC3" s="63"/>
-      <c r="AD3" s="61" t="str">
+      <c r="AA3" s="59"/>
+      <c r="AB3" s="59"/>
+      <c r="AC3" s="60"/>
+      <c r="AD3" s="58" t="str">
         <f>TEXT(AD5,"MMM")</f>
         <v>Mar</v>
       </c>
-      <c r="AE3" s="62"/>
-      <c r="AF3" s="62"/>
-      <c r="AG3" s="62"/>
+      <c r="AE3" s="59"/>
+      <c r="AF3" s="59"/>
+      <c r="AG3" s="59"/>
       <c r="AH3" s="7"/>
-      <c r="AI3" s="61" t="str">
+      <c r="AI3" s="58" t="str">
         <f>TEXT(AI5,"MMM")</f>
         <v>Apr</v>
       </c>
-      <c r="AJ3" s="62"/>
-      <c r="AK3" s="62"/>
-      <c r="AL3" s="63"/>
-      <c r="AM3" s="61" t="str">
+      <c r="AJ3" s="59"/>
+      <c r="AK3" s="59"/>
+      <c r="AL3" s="60"/>
+      <c r="AM3" s="58" t="str">
         <f>TEXT(AM5,"MMM")</f>
         <v>May</v>
       </c>
-      <c r="AN3" s="62"/>
-      <c r="AO3" s="62"/>
-      <c r="AP3" s="63"/>
+      <c r="AN3" s="59"/>
+      <c r="AO3" s="59"/>
+      <c r="AP3" s="60"/>
       <c r="AQ3" s="6" t="str">
         <f>TEXT(AQ5,"MMM")</f>
         <v>Jun</v>
@@ -1253,109 +1249,109 @@
         <v>18</v>
       </c>
       <c r="I5" s="11">
-        <v>45936</v>
+        <v>46301</v>
       </c>
       <c r="J5" s="12">
-        <v>45943</v>
+        <v>46308</v>
       </c>
       <c r="K5" s="13">
-        <v>45950</v>
+        <v>46315</v>
       </c>
       <c r="L5" s="14">
-        <v>45957</v>
+        <v>46322</v>
       </c>
       <c r="M5" s="11">
-        <v>45964</v>
+        <v>46329</v>
       </c>
       <c r="N5" s="12">
-        <v>45971</v>
+        <v>46336</v>
       </c>
       <c r="O5" s="13">
-        <v>45978</v>
+        <v>46343</v>
       </c>
       <c r="P5" s="14">
-        <v>45985</v>
+        <v>46350</v>
       </c>
       <c r="Q5" s="11">
-        <v>45992</v>
+        <v>46357</v>
       </c>
       <c r="R5" s="12">
-        <v>45999</v>
+        <v>46364</v>
       </c>
       <c r="S5" s="13">
-        <v>46006</v>
+        <v>46371</v>
       </c>
       <c r="T5" s="18">
-        <v>46013</v>
+        <v>46378</v>
       </c>
       <c r="U5" s="19">
-        <v>46020</v>
+        <v>46385</v>
       </c>
       <c r="V5" s="11">
-        <v>46027</v>
+        <v>46392</v>
       </c>
       <c r="W5" s="12">
-        <v>46034</v>
+        <v>46399</v>
       </c>
       <c r="X5" s="13">
-        <v>46041</v>
+        <v>46406</v>
       </c>
       <c r="Y5" s="14">
-        <v>46048</v>
+        <v>46413</v>
       </c>
       <c r="Z5" s="11">
-        <v>46055</v>
+        <v>46420</v>
       </c>
       <c r="AA5" s="12">
-        <v>46062</v>
+        <v>46427</v>
       </c>
       <c r="AB5" s="13">
-        <v>46069</v>
+        <v>46434</v>
       </c>
       <c r="AC5" s="14">
-        <v>46076</v>
+        <v>46441</v>
       </c>
       <c r="AD5" s="11">
-        <v>46083</v>
+        <v>46448</v>
       </c>
       <c r="AE5" s="12">
-        <v>46090</v>
+        <v>46455</v>
       </c>
       <c r="AF5" s="13">
-        <v>46097</v>
+        <v>46462</v>
       </c>
       <c r="AG5" s="18">
-        <v>46104</v>
+        <v>46469</v>
       </c>
       <c r="AH5" s="19">
-        <v>46111</v>
+        <v>46476</v>
       </c>
       <c r="AI5" s="11">
-        <v>46118</v>
+        <v>46483</v>
       </c>
       <c r="AJ5" s="12">
-        <v>46125</v>
+        <v>46490</v>
       </c>
       <c r="AK5" s="13">
-        <v>46132</v>
+        <v>46497</v>
       </c>
       <c r="AL5" s="14">
-        <v>46139</v>
+        <v>46504</v>
       </c>
       <c r="AM5" s="11">
-        <v>46146</v>
+        <v>46511</v>
       </c>
       <c r="AN5" s="12">
-        <v>46153</v>
+        <v>46518</v>
       </c>
       <c r="AO5" s="13">
-        <v>46160</v>
+        <v>46525</v>
       </c>
       <c r="AP5" s="14">
-        <v>46167</v>
+        <v>46532</v>
       </c>
       <c r="AQ5" s="20">
-        <v>46174</v>
+        <v>46539</v>
       </c>
       <c r="AS5" s="49" t="s">
         <v>41</v>
@@ -1482,10 +1478,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="30">
-        <v>45936</v>
+        <v>46301</v>
       </c>
       <c r="G8" s="30">
-        <v>45961</v>
+        <v>46326</v>
       </c>
       <c r="H8" s="25"/>
       <c r="I8" s="25">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="AU8" s="56">
         <f>AT8*$D$37</f>
-        <v>135</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1550,10 +1546,10 @@
         <v>0.4</v>
       </c>
       <c r="F9" s="30">
-        <v>45940</v>
+        <v>46312</v>
       </c>
       <c r="G9" s="30">
-        <v>45961</v>
+        <v>46341</v>
       </c>
       <c r="H9" s="24"/>
       <c r="I9" s="25"/>
@@ -1593,15 +1589,15 @@
       <c r="AQ9" s="23"/>
       <c r="AS9" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT9" s="54">
         <f t="shared" ref="AT9:AT26" si="1">AS9*$D$36</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AU9" s="56">
         <f t="shared" ref="AU9:AU26" si="2">AT9*$D$37</f>
-        <v>135</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1615,10 +1611,10 @@
         <v>0.1</v>
       </c>
       <c r="F10" s="30">
-        <v>45945</v>
+        <v>46310</v>
       </c>
       <c r="G10" s="30">
-        <v>45961</v>
+        <v>46326</v>
       </c>
       <c r="H10" s="24"/>
       <c r="I10" s="25"/>
@@ -1666,7 +1662,7 @@
       </c>
       <c r="AU10" s="56">
         <f t="shared" si="2"/>
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1680,10 +1676,10 @@
         <v>0.05</v>
       </c>
       <c r="F11" s="30">
-        <v>45955</v>
+        <v>46320</v>
       </c>
       <c r="G11" s="30">
-        <v>45961</v>
+        <v>46326</v>
       </c>
       <c r="H11" s="24"/>
       <c r="I11" s="25"/>
@@ -1797,12 +1793,8 @@
       </c>
       <c r="D13" s="33"/>
       <c r="E13" s="26"/>
-      <c r="F13" s="30">
-        <v>45945</v>
-      </c>
-      <c r="G13" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
       <c r="H13" s="24"/>
       <c r="I13" s="25"/>
       <c r="J13" s="25"/>
@@ -1841,15 +1833,15 @@
       <c r="AQ13" s="23"/>
       <c r="AS13" s="8">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AT13" s="54">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="AU13" s="56">
         <f t="shared" si="2"/>
-        <v>495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1858,12 +1850,8 @@
       </c>
       <c r="D14" s="33"/>
       <c r="E14" s="26"/>
-      <c r="F14" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G14" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
       <c r="H14" s="24"/>
       <c r="I14" s="25"/>
       <c r="J14" s="25"/>
@@ -1902,15 +1890,15 @@
       <c r="AQ14" s="23"/>
       <c r="AS14" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT14" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU14" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1919,12 +1907,8 @@
       </c>
       <c r="D15" s="33"/>
       <c r="E15" s="26"/>
-      <c r="F15" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G15" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
       <c r="H15" s="24"/>
       <c r="I15" s="25"/>
       <c r="J15" s="25"/>
@@ -1963,15 +1947,15 @@
       <c r="AQ15" s="23"/>
       <c r="AS15" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT15" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU15" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1980,12 +1964,8 @@
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="26"/>
-      <c r="F16" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G16" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
       <c r="H16" s="24"/>
       <c r="I16" s="25"/>
       <c r="J16" s="25"/>
@@ -2024,15 +2004,15 @@
       <c r="AQ16" s="23"/>
       <c r="AS16" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT16" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU16" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="3:47" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2098,12 +2078,8 @@
       </c>
       <c r="D18" s="33"/>
       <c r="E18" s="26"/>
-      <c r="F18" s="30">
-        <v>45945</v>
-      </c>
-      <c r="G18" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
       <c r="H18" s="24"/>
       <c r="I18" s="25"/>
       <c r="J18" s="25"/>
@@ -2142,15 +2118,15 @@
       <c r="AQ18" s="23"/>
       <c r="AS18" s="8">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AT18" s="54">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="AU18" s="56">
         <f t="shared" si="2"/>
-        <v>495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2159,12 +2135,8 @@
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="26"/>
-      <c r="F19" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G19" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
       <c r="H19" s="24"/>
       <c r="I19" s="25"/>
       <c r="J19" s="25"/>
@@ -2203,15 +2175,15 @@
       <c r="AQ19" s="23"/>
       <c r="AS19" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT19" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU19" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2220,12 +2192,8 @@
       </c>
       <c r="D20" s="33"/>
       <c r="E20" s="26"/>
-      <c r="F20" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G20" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
       <c r="H20" s="24"/>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
@@ -2264,15 +2232,15 @@
       <c r="AQ20" s="23"/>
       <c r="AS20" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT20" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU20" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2281,12 +2249,8 @@
       </c>
       <c r="D21" s="33"/>
       <c r="E21" s="26"/>
-      <c r="F21" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G21" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
       <c r="H21" s="24"/>
       <c r="I21" s="25"/>
       <c r="J21" s="25"/>
@@ -2325,15 +2289,15 @@
       <c r="AQ21" s="23"/>
       <c r="AS21" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT21" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU21" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="3:47" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2399,12 +2363,8 @@
       </c>
       <c r="D23" s="33"/>
       <c r="E23" s="26"/>
-      <c r="F23" s="30">
-        <v>45945</v>
-      </c>
-      <c r="G23" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
       <c r="H23" s="24"/>
       <c r="I23" s="25"/>
       <c r="J23" s="25"/>
@@ -2443,15 +2403,15 @@
       <c r="AQ23" s="23"/>
       <c r="AS23" s="8">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AT23" s="54">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="AU23" s="56">
         <f t="shared" si="2"/>
-        <v>495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2460,12 +2420,8 @@
       </c>
       <c r="D24" s="33"/>
       <c r="E24" s="26"/>
-      <c r="F24" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G24" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
       <c r="H24" s="24"/>
       <c r="I24" s="25"/>
       <c r="J24" s="25"/>
@@ -2504,15 +2460,15 @@
       <c r="AQ24" s="23"/>
       <c r="AS24" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT24" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU24" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2521,12 +2477,8 @@
       </c>
       <c r="D25" s="33"/>
       <c r="E25" s="26"/>
-      <c r="F25" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G25" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
       <c r="H25" s="24"/>
       <c r="I25" s="25"/>
       <c r="J25" s="25"/>
@@ -2565,15 +2517,15 @@
       <c r="AQ25" s="23"/>
       <c r="AS25" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT25" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU25" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="3:47" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2582,12 +2534,8 @@
       </c>
       <c r="D26" s="33"/>
       <c r="E26" s="26"/>
-      <c r="F26" s="30">
-        <v>45962</v>
-      </c>
-      <c r="G26" s="30">
-        <v>46022</v>
-      </c>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
       <c r="H26" s="24"/>
       <c r="I26" s="25"/>
       <c r="J26" s="25"/>
@@ -2626,15 +2574,15 @@
       <c r="AQ26" s="23"/>
       <c r="AS26" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AT26" s="54">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AU26" s="56">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="3:47" x14ac:dyDescent="0.3">
@@ -2660,50 +2608,50 @@
       <c r="C30" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="59" t="s">
+      <c r="D30" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="E30" s="59"/>
-      <c r="F30" s="60"/>
+      <c r="E30" s="63"/>
+      <c r="F30" s="64"/>
       <c r="AS30" s="52">
         <f>SUM(AS8:AS26)</f>
-        <v>113</v>
+        <v>9</v>
       </c>
       <c r="AT30" s="55">
         <f>SUM(AT8:AT26)</f>
-        <v>339</v>
+        <v>27</v>
       </c>
       <c r="AU30" s="57">
         <f>SUM(AU8:AU26)</f>
-        <v>5085</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" spans="3:47" x14ac:dyDescent="0.3">
       <c r="C31" s="43"/>
-      <c r="D31" s="59" t="s">
+      <c r="D31" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="E31" s="59"/>
-      <c r="F31" s="60"/>
+      <c r="E31" s="63"/>
+      <c r="F31" s="64"/>
     </row>
     <row r="32" spans="3:47" x14ac:dyDescent="0.3">
       <c r="C32" s="43"/>
-      <c r="D32" s="59" t="s">
+      <c r="D32" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="E32" s="59"/>
-      <c r="F32" s="60"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="64"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
     <row r="33" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C33" s="43"/>
-      <c r="D33" s="59" t="s">
+      <c r="D33" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="59"/>
-      <c r="F33" s="60"/>
+      <c r="E33" s="63"/>
+      <c r="F33" s="64"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -2746,7 +2694,7 @@
         <v>36</v>
       </c>
       <c r="D37" s="47">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E37" s="38" t="s">
         <v>34</v>
@@ -2776,20 +2724,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="V3:Y3"/>
+    <mergeCell ref="Z3:AC3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="D30:F30"/>
     <mergeCell ref="AI3:AL3"/>
     <mergeCell ref="AM3:AP3"/>
     <mergeCell ref="I3:L3"/>
     <mergeCell ref="M3:P3"/>
     <mergeCell ref="Q3:T3"/>
     <mergeCell ref="AD3:AG3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="V3:Y3"/>
-    <mergeCell ref="Z3:AC3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="D33:F33"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="E8:E26">

</xml_diff>